<commit_message>
Complete Phase 7 SQL analytics and update project documentation
</commit_message>
<xml_diff>
--- a/sql/Phase 6_analytics requirements & reporting design/02_Phase_6_KPI_and_Data_Mapping.xlsx
+++ b/sql/Phase 6_analytics requirements & reporting design/02_Phase_6_KPI_and_Data_Mapping.xlsx
@@ -548,7 +548,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Completed-order eligibility selected; validate monetary field/grain against SQL before implementation; refund netting undefined.</t>
+          <t>Completed-order sales basis and line-level monetary aggregation validated in SQL 7.3/7.4: AED 26,870. Use one grain consistently; do not mix header and line amounts. Refund netting remains undefined.</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Selected completed-order basis: AED 1,791.33; numerator and denominator must match.</t>
+          <t>Selected completed-order basis validated: AED 26,870 / 15 = AED 1,791.33.</t>
         </is>
       </c>
     </row>
@@ -770,7 +770,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>AED 7,603 estimated using current cost; not historical accounting profit.</t>
+          <t>SQL 7.12 validated AED 5,360 (AED 26,870 eligible sales less AED 21,510 estimated current product cost). Earlier AED 7,603 benchmark is superseded; AED 2,243 variance remains unexplained and is not an adjustment. Not historical/audited profit.</t>
         </is>
       </c>
     </row>
@@ -807,7 +807,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Estimated only; validate sales/cost grain and measure aggregation; current product cost is not historical.</t>
+          <t>SQL 7.12 validated estimated margin: 19.95% (AED 5,360 / AED 26,870). Current product cost only; label as estimated and guard zero sales.</t>
         </is>
       </c>
     </row>
@@ -844,7 +844,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Completed-order basis selected; 28 units across all statuses previously validated.</t>
+          <t>Completed-order basis validated: 21 units in 15 completed orders. The earlier 28-unit figure refers to all statuses and must not be used for this completed-order KPI.</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Completed-order basis selected; validate line_total aggregation and relationship behavior against SQL.</t>
+          <t>Completed-order product sales validated in SQL 7.6: 14 products, 21 units, AED 26,870. Category totals reconcile in SQL 7.8.</t>
         </is>
       </c>
     </row>
@@ -918,7 +918,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>15 customers have orders overall; 11 have completed purchases. Define metric label carefully.</t>
+          <t>11 customers with completed purchases; 15 customers have orders overall. Completed-order customer analysis validated in SQL 7.9.</t>
         </is>
       </c>
     </row>
@@ -955,7 +955,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Current snapshot only.</t>
+          <t>Current snapshot; stored available_stock reconciles to current_stock − reserved_stock across 19 records (SQL 7.11).</t>
         </is>
       </c>
     </row>
@@ -992,7 +992,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Selected operational rule: available_stock at or below reorder_level; 3 rows previously validated.</t>
+          <t>Selected operational rule validated in SQL 7.11: 3 product/warehouse rows at or below reorder level.</t>
         </is>
       </c>
     </row>
@@ -1610,7 +1610,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Confirm composition, discounts, tax and shipping.</t>
+          <t>SQL 7.3/7.4 reconciled completed-order sales at AED 26,870 using line_total; order_total is a distinct header-grain field and must not be mixed with line totals.</t>
         </is>
       </c>
     </row>
@@ -1708,7 +1708,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Not yet verified</t>
+          <t>commerce.product.cost_price</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -1718,7 +1718,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Current cost field verified as commerce.product.cost_price; historical cost unavailable in the reviewed schema.</t>
+          <t>Current cost field cost_price verified in SQL 7.12; historical cost unavailable. Estimated profitability only.</t>
         </is>
       </c>
     </row>
@@ -1961,7 +1961,7 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Validated against quantity × unit_price − discount_amount; avoid double counting with order_total.</t>
+          <t>SQL 7.3/7.4/7.12 validated completed-order line_total aggregation: AED 26,870. Avoid double counting with order_total.</t>
         </is>
       </c>
     </row>
@@ -2220,7 +2220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="37" customWidth="1" min="1" max="1"/>
@@ -2243,7 +2243,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Phase 6 documentation closed after consistency review; SQL/Power BI implementation and acceptance testing pending.</t>
+          <t>Phase 6 documentation revised after SQL 7.12 profitability validation; SQL/Power BI implementation and acceptance testing pending.</t>
         </is>
       </c>
     </row>
@@ -2340,6 +2340,18 @@
       <c r="B10" t="inlineStr">
         <is>
           <t>Reviewed schema, columns and listed FK paths documented; data completeness, KPI implementation and acceptance remain unverified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Profitability validation</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>SQL 7.12 validated: AED 26,870 eligible sales; AED 21,510 estimated current product cost; AED 5,360 estimated gross profit; 19.95% estimated margin. Prior AED 7,603 benchmark is superseded; AED 2,243 variance remains unexplained and is not an adjustment.</t>
         </is>
       </c>
     </row>
@@ -2378,7 +2390,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Phase 6 documentation closed; implementation and acceptance testing pending.</t>
+          <t>Phase 6 documentation revised after SQL 7.12 profitability validation; implementation and acceptance testing pending.</t>
         </is>
       </c>
     </row>
@@ -2438,7 +2450,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Estimated Gross Profit = eligible completed-order sales less estimated product cost using current product costs. Label profit and margin as estimated; not historical or audited.</t>
+          <t>Estimated Gross Profit = eligible completed-order sales less estimated product cost using current product costs. SQL 7.12 validated: AED 26,870 sales − AED 21,510 estimated cost = AED 5,360 estimated gross profit; estimated margin 19.95%. Earlier AED 7,603 benchmark is superseded; AED 2,243 variance remains unexplained and is not an adjustment. Not historical or audited.</t>
         </is>
       </c>
     </row>
@@ -2486,7 +2498,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Final cross-document consistency review completed; Phase 6 documentation closed. Power BI implementation is subsequent work.</t>
+          <t>Phase 6 documentation updated after SQL 7.12 profitability validation. Confirm all three documents contain matching values; Power BI implementation and acceptance testing remain subsequent work.</t>
         </is>
       </c>
     </row>
@@ -2498,7 +2510,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Validate Total Sales monetary basis/grain; define Completion Rate denominator before implementation; reconcile KPI outputs to independent SQL; test relationships, slicers and acceptance criteria.</t>
+          <t>Total Sales basis/grain and profitability reconciled through SQL 7.12; Completion Rate denominator remains undefined. Reconcile KPI outputs to independent SQL and test relationships, slicers and acceptance criteria.</t>
         </is>
       </c>
     </row>

</xml_diff>